<commit_message>
date function call implementation still in progress
</commit_message>
<xml_diff>
--- a/2-Tests/Lexerow.Core.Tests/10-ExcelFiles/OnExcelIfThenDateOk.xlsx
+++ b/2-Tests/Lexerow.Core.Tests/10-ExcelFiles/OnExcelIfThenDateOk.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29426"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/a990f455bb745add/ProjetsDev/10-Pierlam/Lexerow/Dev/Lexerow/2-Tests/Lexerow.Core.Tests/10-ExcelFiles/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="44" documentId="11_2B8C63A238C272CACCFC3B895DC533011B7D74F5" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{40F5A0C2-4210-4529-B340-A657BBDBB170}"/>
+  <xr:revisionPtr revIDLastSave="57" documentId="11_2B8C63A238C272CACCFC3B895DC533011B7D74F5" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B1395031-F4FD-4DAD-89FB-F677007FEE68}"/>
   <bookViews>
     <workbookView xWindow="4455" yWindow="4470" windowWidth="18900" windowHeight="10515" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="7">
   <si>
     <t>date</t>
   </si>
@@ -39,19 +39,19 @@
     <t>dateTime</t>
   </si>
   <si>
-    <t>If A.Cell &lt;= 10 Then A.Cell=Date(2025, 11, 30)</t>
-  </si>
-  <si>
     <t>blabla</t>
+  </si>
+  <si>
+    <t>If A.Cell &lt;= 10 Then B.Cell=Date(2025, 11, 30)</t>
+  </si>
+  <si>
+    <t>nothing</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="#,##0.00\ &quot;€&quot;"/>
-  </numFmts>
   <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -87,9 +87,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="21" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="14" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
@@ -108,6 +107,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -373,7 +376,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D5"/>
+  <dimension ref="A1:D6"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="18.28515625" customWidth="1"/>
@@ -386,7 +389,7 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
@@ -394,12 +397,14 @@
         <v>10</v>
       </c>
       <c r="B2" t="s">
-        <v>5</v>
-      </c>
-      <c r="C2" s="4">
+        <v>4</v>
+      </c>
+      <c r="C2" s="3">
         <v>45991</v>
       </c>
-      <c r="D2" s="1"/>
+      <c r="D2">
+        <v>1</v>
+      </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3">
@@ -408,31 +413,53 @@
       <c r="B3" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="C3" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="D3" s="1"/>
+      <c r="D3">
+        <v>2</v>
+      </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A4" s="3">
+      <c r="A4" s="2">
         <v>0.15306712962962962</v>
       </c>
       <c r="B4" t="s">
         <v>2</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="C4" s="2" t="s">
         <v>2</v>
       </c>
+      <c r="D4">
+        <v>3</v>
+      </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A5" s="2">
+      <c r="A5" s="1">
         <v>43223.521354166667</v>
       </c>
       <c r="B5" t="s">
         <v>3</v>
       </c>
-      <c r="C5" s="2" t="s">
+      <c r="C5" s="1" t="s">
         <v>3</v>
+      </c>
+      <c r="D5">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A6">
+        <v>15</v>
+      </c>
+      <c r="B6" t="s">
+        <v>6</v>
+      </c>
+      <c r="C6" t="s">
+        <v>6</v>
+      </c>
+      <c r="D6">
+        <v>5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>